<commit_message>
Update demo portfolio with realistic sample data
- 3 family members: Siddiq, Zayyan, Fahima
- Real asset types: ETFs, Stocks, Crypto, Gold, Silver, Cash
- Combined Summary sheet included
- Matches exact app export format for seamless import
- Updated README with detailed demo breakdown
</commit_message>
<xml_diff>
--- a/samples/demo_portfolio.xlsx
+++ b/samples/demo_portfolio.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ahmed" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fatima" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siddiq" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zayyan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fahima" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,12 +416,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -430,14 +432,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Zakat Calculator - Ahmed</t>
+          <t>Zakat Calculator - Siddiq</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Exported: 11/03/2026, 14:30:00</t>
+          <t>Exported: 3/2/2026, 5:28:29 PM</t>
         </is>
       </c>
     </row>
@@ -500,28 +502,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VWCE.DE</t>
+          <t>IE0009JOT9U1.SG</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World</t>
+          <t>iShares Physical Gold EUR Hedge</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D7" t="n">
-        <v>105.2</v>
+        <v>72.45999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>118.45</v>
+        <v>93.84</v>
       </c>
       <c r="F7" t="n">
-        <v>5922.5</v>
+        <v>5255.04</v>
       </c>
       <c r="G7" t="n">
-        <v>662.5</v>
+        <v>1197.28</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -532,28 +534,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ISAC.L</t>
+          <t>PPFD.SG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>iShares MSCI ACWI</t>
+          <t>iShares Physical Silver ETC</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>62.3</v>
+        <v>89.43000000000001</v>
       </c>
       <c r="E8" t="n">
-        <v>68.90000000000001</v>
+        <v>73.45</v>
       </c>
       <c r="F8" t="n">
-        <v>6890</v>
+        <v>146.9</v>
       </c>
       <c r="G8" t="n">
-        <v>660</v>
+        <v>-31.96</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -613,28 +615,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MBG.DE</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Group</t>
+          <t>Amazon.com, Inc.</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>58.5</v>
+        <v>168.76</v>
       </c>
       <c r="E12" t="n">
-        <v>72.3</v>
+        <v>177.55</v>
       </c>
       <c r="F12" t="n">
-        <v>2169</v>
+        <v>532.64</v>
       </c>
       <c r="G12" t="n">
-        <v>414</v>
+        <v>26.36</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -645,28 +647,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SAP.DE</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>145</v>
+        <v>170.92</v>
       </c>
       <c r="E13" t="n">
-        <v>210.5</v>
+        <v>226.59</v>
       </c>
       <c r="F13" t="n">
-        <v>3157.5</v>
+        <v>453.18</v>
       </c>
       <c r="G13" t="n">
-        <v>982.5</v>
+        <v>111.34</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -674,80 +676,127 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E14" t="n">
+        <v>154.94</v>
+      </c>
+      <c r="F14" t="n">
+        <v>619.74</v>
+      </c>
+      <c r="G14" t="n">
+        <v>139.74</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15">
-        <f>== Crypto ===</f>
-        <v/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Procter &amp; Gamble Company (The)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>149.42</v>
+      </c>
+      <c r="E15" t="n">
+        <v>141.03</v>
+      </c>
+      <c r="F15" t="n">
+        <v>564.11</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-33.57</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Symbol</t>
+          <t>TPE.DE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Avg Price</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Current Price</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Profit</t>
-        </is>
+          <t>PVA TePla AG</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>23</v>
+      </c>
+      <c r="D16" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="E16" t="n">
+        <v>27.52</v>
+      </c>
+      <c r="F16" t="n">
+        <v>632.96</v>
+      </c>
+      <c r="G16" t="n">
+        <v>29.21</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>EUR</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BTC-USD</t>
+          <t>SHL.DE</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>Siemens Healthineers AG</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.15</v>
+        <v>10</v>
       </c>
       <c r="D17" t="n">
-        <v>42000</v>
+        <v>53.82</v>
       </c>
       <c r="E17" t="n">
-        <v>68500</v>
+        <v>41.24</v>
       </c>
       <c r="F17" t="n">
-        <v>10275</v>
+        <v>412.4</v>
       </c>
       <c r="G17" t="n">
-        <v>3975</v>
+        <v>-125.8</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -758,28 +807,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH-USD</t>
+          <t>ZETA</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Zeta Global Holdings Corp.</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2.5</v>
+        <v>25</v>
       </c>
       <c r="D18" t="n">
-        <v>2200</v>
+        <v>16.5</v>
       </c>
       <c r="E18" t="n">
-        <v>3850</v>
+        <v>14.79</v>
       </c>
       <c r="F18" t="n">
-        <v>9625</v>
+        <v>369.86</v>
       </c>
       <c r="G18" t="n">
-        <v>4125</v>
+        <v>-42.64</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -790,259 +839,227 @@
     <row r="19"/>
     <row r="20">
       <c r="A20">
+        <f>== Crypto ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Avg Price</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GB00BNRRFY34.SG</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CoinShares Physical Staked Sola</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>38</v>
+      </c>
+      <c r="D22" t="n">
+        <v>7.78</v>
+      </c>
+      <c r="E22" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="F22" t="n">
+        <v>324.54</v>
+      </c>
+      <c r="G22" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24">
         <f>== Physical Gold ===</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Weight (g)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Karat</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Buy Price/g</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Current Price/g</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Gold Chain 22K</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>25</v>
-      </c>
-      <c r="C22" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>coins</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>51</v>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>22K</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>55</v>
-      </c>
-      <c r="E22" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="F22" t="n">
-        <v>1962.5</v>
-      </c>
-      <c r="G22" t="n">
-        <v>587.5</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Gold Coins</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>50</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>22K</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>52</v>
-      </c>
-      <c r="E23" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="F23" t="n">
-        <v>3925</v>
-      </c>
-      <c r="G23" t="n">
-        <v>1325</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Wedding Ring</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>8</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>22K</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>48</v>
-      </c>
-      <c r="E24" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="F24" t="n">
-        <v>628</v>
-      </c>
-      <c r="G24" t="n">
-        <v>244</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26">
-        <f>== Physical Silver ===</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Weight (g)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Purity (%)</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Buy Price/g</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Current Price/g</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Profit</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-    </row>
+      <c r="D26" t="n">
+        <v>63</v>
+      </c>
+      <c r="E26" t="n">
+        <v>133.56</v>
+      </c>
+      <c r="F26" t="n">
+        <v>6811.47</v>
+      </c>
+      <c r="G26" t="n">
+        <v>3598.47</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Silver Bars</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>500</v>
-      </c>
-      <c r="C28" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F28" t="n">
-        <v>475</v>
-      </c>
-      <c r="G28" t="n">
-        <v>150</v>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30">
+      <c r="A28">
         <f>== Cash &amp; Other ===</f>
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>n26</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>8600</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
+          <t>kisna</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1000</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>EUR</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Savings Account (Deutsche Bank)</t>
+          <t>revolut</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>15000</v>
+        <v>250</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1053,11 +1070,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Emergency Fund</t>
+          <t>india</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>5000</v>
+        <v>300</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1065,53 +1082,53 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Cash at Home</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>800</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36">
+    <row r="34"/>
+    <row r="35">
+      <c r="A35">
         <f>== Liabilities ===</f>
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
+          <t>rent</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1040</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>EUR</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Car Loan (Monthly)</t>
+          <t>expense</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>350</v>
+        <v>1000</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1119,16 +1136,202 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Credit Card Balance</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1200</v>
-      </c>
-      <c r="C39" t="inlineStr">
+    <row r="39"/>
+    <row r="40">
+      <c r="A40">
+        <f>== Summary ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ETFs</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5401.94</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>324.54</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Stocks</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>3584.89</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Physical Gold</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>6811.47</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Physical Silver</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Cash &amp; Other</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>10150</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>26272.84</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Liabilities</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2040</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Net Wealth</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>24232.84</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Nisab Threshold</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>12745.84</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Above Nisab?</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Zakat Due (2.5%)</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>605.8200000000001</v>
+      </c>
+      <c r="C53" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
@@ -1145,12 +1348,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -1161,14 +1364,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Zakat Calculator - Fatima</t>
+          <t>Zakat Calculator - Zayyan</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Exported: 11/03/2026, 14:30:00</t>
+          <t>Exported: 3/2/2026, 5:28:29 PM</t>
         </is>
       </c>
     </row>
@@ -1182,34 +1385,553 @@
     <row r="4"/>
     <row r="5">
       <c r="A5">
+        <f>== ETFs ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Avg Price</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IE0009JOT9U1.SG</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>iShares Physical Gold EUR Hedge</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" t="n">
+        <v>81.68000000000001</v>
+      </c>
+      <c r="E7" t="n">
+        <v>93.84</v>
+      </c>
+      <c r="F7" t="n">
+        <v>938.4</v>
+      </c>
+      <c r="G7" t="n">
+        <v>121.6</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ISWD.SW</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>iSh MSCI Wld Islamic USD D</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>52.16</v>
+      </c>
+      <c r="F8" t="n">
+        <v>521.63</v>
+      </c>
+      <c r="G8" t="n">
+        <v>29.59</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10">
         <f>== Physical Gold ===</f>
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Weight (g)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Karat</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Buy Price/g</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Current Price/g</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>jewels</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>60</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>110</v>
+      </c>
+      <c r="E12" t="n">
+        <v>133.56</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8013.5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1413.5</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14">
+        <f>== Physical Silver ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Weight (g)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Purity (%)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Buy Price/g</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Current Price/g</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>jewels</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>201</v>
+      </c>
+      <c r="C16" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F16" t="n">
+        <v>483.93</v>
+      </c>
+      <c r="G16" t="n">
+        <v>282.93</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18">
+        <f>== Summary ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ETFs</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1460.03</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Stocks</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Physical Gold</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>8013.5</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Physical Silver</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>483.93</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cash &amp; Other</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>9957.450000000001</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Liabilities</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Net Wealth</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>9957.450000000001</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nisab Threshold</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>12745.84</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Above Nisab?</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Zakat Due (2.5%)</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Zakat Calculator - Fahima</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exported: 3/2/2026, 5:28:29 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Currency: EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5">
+        <f>== ETFs ===</f>
+        <v/>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Symbol</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Weight (g)</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Karat</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Buy Price/g</t>
+          <t>Avg Price</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Current Price/g</t>
+          <t>Current Price</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1231,28 +1953,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gold Necklace Set</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>22K</t>
-        </is>
+          <t>IE0009JOT9U1.SG</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>iShares Physical Gold EUR Hedge</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>24</v>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>81.93000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>78.5</v>
+        <v>93.84</v>
       </c>
       <c r="F7" t="n">
-        <v>3532.5</v>
+        <v>2252.16</v>
       </c>
       <c r="G7" t="n">
-        <v>1282.5</v>
+        <v>285.84</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1260,151 +1982,161 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Gold Bangles (4 pcs)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>80</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>22K</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>53</v>
-      </c>
-      <c r="E8" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>6280</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2040</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Gold Earrings</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>12</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>22K</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>56</v>
-      </c>
-      <c r="E9" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="F9" t="n">
-        <v>942</v>
-      </c>
-      <c r="G9" t="n">
-        <v>270</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
+      <c r="A9">
+        <f>== Physical Gold ===</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mahr Gold Set</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>100</v>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Weight (g)</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Karat</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Buy Price/g</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Current Price/g</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>jewels</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>750</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>22K</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>45</v>
-      </c>
-      <c r="E10" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="F10" t="n">
-        <v>7850</v>
-      </c>
-      <c r="G10" t="n">
-        <v>3350</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12">
-        <f>== Cash &amp; Other ===</f>
+      <c r="D11" t="n">
+        <v>89</v>
+      </c>
+      <c r="E11" t="n">
+        <v>133.56</v>
+      </c>
+      <c r="F11" t="n">
+        <v>100168.75</v>
+      </c>
+      <c r="G11" t="n">
+        <v>33418.75</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13">
+        <f>== Physical Silver ===</f>
         <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Personal Savings</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>8500</v>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Weight (g)</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>Purity (%)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Buy Price/g</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Current Price/g</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Currency</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fixed Deposit</t>
+          <t>jewels</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C15" t="inlineStr">
+        <v>20</v>
+      </c>
+      <c r="C15" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F15" t="n">
+        <v>48.15</v>
+      </c>
+      <c r="G15" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
@@ -1413,7 +2145,7 @@
     <row r="16"/>
     <row r="17">
       <c r="A17">
-        <f>== Liabilities ===</f>
+        <f>== Cash &amp; Other ===</f>
         <v/>
       </c>
     </row>
@@ -1437,13 +2169,372 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Personal Loan</t>
+          <t>n26</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2000</v>
+        <v>1885</v>
       </c>
       <c r="C19" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21">
+        <f>== Summary ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ETFs</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2252.16</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Stocks</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Physical Gold</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>100168.75</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Physical Silver</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>48.15</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cash &amp; Other</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1885</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>104354.06</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Liabilities</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Net Wealth</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>104354.06</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Nisab Threshold</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>12745.84</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Above Nisab?</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Zakat Due (2.5%)</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2608.85</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Combined Zakat Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exported: 3/2/2026, 5:28:29 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Currency: EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Net Wealth</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Zakat Due</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Above Nisab?</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Siddiq</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>24232.84</v>
+      </c>
+      <c r="C6" t="n">
+        <v>605.8200000000001</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Zayyan</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>9957.450000000001</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fahima</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>104354.06</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2608.85</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>138544.35</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3214.67</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>

<commit_message>
Update demo portfolio Excel file with new data
</commit_message>
<xml_diff>
--- a/samples/demo_portfolio.xlsx
+++ b/samples/demo_portfolio.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Siddiq" sheetId="1" r:id="rId1"/>
-    <sheet name="Zayyan" sheetId="2" r:id="rId2"/>
-    <sheet name="Fahima" sheetId="3" r:id="rId3"/>
+    <sheet name="Father" sheetId="1" r:id="rId1"/>
+    <sheet name="Son" sheetId="2" r:id="rId2"/>
+    <sheet name="Mother" sheetId="3" r:id="rId3"/>
     <sheet name="Combined Summary" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
@@ -402,7 +402,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H53"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
     <col min="2" max="2" width="33.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
@@ -414,12 +414,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Zakat Calculator - Siddiq</v>
+        <v>Zakat Calculator - Father</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Exported: 3/2/2026, 5:28:29 PM</v>
+        <v>Exported: 3/13/2026, 3:54:02 PM</v>
       </c>
     </row>
     <row r="3">
@@ -816,7 +816,7 @@
         <v>coins</v>
       </c>
       <c r="B26">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C26" t="str">
         <v>22K</v>
@@ -828,10 +828,10 @@
         <v>133.5583333333333</v>
       </c>
       <c r="F26">
-        <v>6811.4749999999985</v>
+        <v>2671.166666666666</v>
       </c>
       <c r="G26">
-        <v>3598.4749999999985</v>
+        <v>1411.166666666666</v>
       </c>
       <c r="H26" t="str">
         <v>EUR</v>
@@ -989,7 +989,7 @@
         <v>Physical Gold</v>
       </c>
       <c r="B45">
-        <v>6811.4749999999985</v>
+        <v>2671.166666666666</v>
       </c>
       <c r="C45" t="str">
         <v>EUR</v>
@@ -1022,7 +1022,7 @@
         <v>Total Assets</v>
       </c>
       <c r="B48">
-        <v>26272.841099999998</v>
+        <v>22132.532766666664</v>
       </c>
       <c r="C48" t="str">
         <v>EUR</v>
@@ -1044,7 +1044,7 @@
         <v>Net Wealth</v>
       </c>
       <c r="B50">
-        <v>24232.841099999998</v>
+        <v>20092.532766666664</v>
       </c>
       <c r="C50" t="str">
         <v>EUR</v>
@@ -1055,7 +1055,7 @@
         <v>Nisab Threshold</v>
       </c>
       <c r="B51">
-        <v>12745.836</v>
+        <v>12468.5244</v>
       </c>
       <c r="C51" t="str">
         <v>EUR</v>
@@ -1077,7 +1077,7 @@
         <v>Zakat Due (2.5%)</v>
       </c>
       <c r="B53">
-        <v>605.8210275</v>
+        <v>502.3133191666666</v>
       </c>
       <c r="C53" t="str">
         <v>EUR</v>
@@ -1094,7 +1094,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H31"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
     <col min="2" max="2" width="33.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
@@ -1106,12 +1106,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Zakat Calculator - Zayyan</v>
+        <v>Zakat Calculator - Son</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Exported: 3/2/2026, 5:28:29 PM</v>
+        <v>Exported: 3/13/2026, 3:54:02 PM</v>
       </c>
     </row>
     <row r="3">
@@ -1436,7 +1436,7 @@
         <v>Nisab Threshold</v>
       </c>
       <c r="B29">
-        <v>12745.836</v>
+        <v>12468.5244</v>
       </c>
       <c r="C29" t="str">
         <v>EUR</v>
@@ -1475,24 +1475,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H34"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
     <col min="2" max="2" width="33.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="19.83203125" customWidth="1"/>
+    <col min="6" max="6" width="19.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Zakat Calculator - Fahima</v>
+        <v>Zakat Calculator - Mother</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Exported: 3/2/2026, 5:28:29 PM</v>
+        <v>Exported: 3/13/2026, 3:54:02 PM</v>
       </c>
     </row>
     <row r="3">
@@ -1593,7 +1593,7 @@
         <v>jewels</v>
       </c>
       <c r="B11">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="C11" t="str">
         <v>22K</v>
@@ -1605,10 +1605,10 @@
         <v>133.5583333333333</v>
       </c>
       <c r="F11">
-        <v>100168.74999999999</v>
+        <v>33389.58333333333</v>
       </c>
       <c r="G11">
-        <v>33418.74999999998</v>
+        <v>11139.583333333327</v>
       </c>
       <c r="H11" t="str">
         <v>EUR</v>
@@ -1752,7 +1752,7 @@
         <v>Physical Gold</v>
       </c>
       <c r="B26">
-        <v>100168.74999999999</v>
+        <v>33389.58333333333</v>
       </c>
       <c r="C26" t="str">
         <v>EUR</v>
@@ -1785,7 +1785,7 @@
         <v>Total Assets</v>
       </c>
       <c r="B29">
-        <v>104354.0618</v>
+        <v>37574.89513333333</v>
       </c>
       <c r="C29" t="str">
         <v>EUR</v>
@@ -1807,7 +1807,7 @@
         <v>Net Wealth</v>
       </c>
       <c r="B31">
-        <v>104354.0618</v>
+        <v>37574.89513333333</v>
       </c>
       <c r="C31" t="str">
         <v>EUR</v>
@@ -1818,7 +1818,7 @@
         <v>Nisab Threshold</v>
       </c>
       <c r="B32">
-        <v>12745.836</v>
+        <v>12468.5244</v>
       </c>
       <c r="C32" t="str">
         <v>EUR</v>
@@ -1840,7 +1840,7 @@
         <v>Zakat Due (2.5%)</v>
       </c>
       <c r="B34">
-        <v>2608.851545</v>
+        <v>939.3723783333334</v>
       </c>
       <c r="C34" t="str">
         <v>EUR</v>
@@ -1871,7 +1871,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Exported: 3/2/2026, 5:28:29 PM</v>
+        <v>Exported: 3/13/2026, 3:54:02 PM</v>
       </c>
     </row>
     <row r="3">
@@ -1898,13 +1898,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Siddiq</v>
+        <v>Father</v>
       </c>
       <c r="B6">
-        <v>24232.841099999998</v>
+        <v>20092.532766666664</v>
       </c>
       <c r="C6">
-        <v>605.8210275</v>
+        <v>502.3133191666666</v>
       </c>
       <c r="D6" t="str">
         <v>Yes</v>
@@ -1915,7 +1915,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Zayyan</v>
+        <v>Son</v>
       </c>
       <c r="B7">
         <v>9957.451377946998</v>
@@ -1932,13 +1932,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Fahima</v>
+        <v>Mother</v>
       </c>
       <c r="B8">
-        <v>104354.0618</v>
+        <v>37574.89513333333</v>
       </c>
       <c r="C8">
-        <v>2608.851545</v>
+        <v>939.3723783333334</v>
       </c>
       <c r="D8" t="str">
         <v>Yes</v>
@@ -1952,10 +1952,10 @@
         <v>TOTAL</v>
       </c>
       <c r="B10">
-        <v>138544.354277947</v>
+        <v>67624.879277947</v>
       </c>
       <c r="C10">
-        <v>3214.6725725</v>
+        <v>1441.6856975</v>
       </c>
       <c r="D10" t="str">
         <v/>

</xml_diff>